<commit_message>
Correction of temporary handling of co-located cases in case_setup.py + minor testcases fix
</commit_message>
<xml_diff>
--- a/testcases.xlsx
+++ b/testcases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\energinet.local\endk_funktion\Dynsim\13_Medarbejdermapper\CVL\MTB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0766EC9-A7A5-4765-A13C-18FF12E68EBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{200E89C6-411A-4F33-AC6B-03B1B8EF80A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2440" yWindow="14290" windowWidth="29020" windowHeight="17500" tabRatio="822" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4667,7 +4667,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="413">
+  <cellXfs count="412">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -5743,20 +5743,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -9256,102 +9253,102 @@
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="334"/>
       <c r="B2" s="334"/>
-      <c r="C2" s="410" t="s">
+      <c r="C2" s="408" t="s">
         <v>848</v>
       </c>
-      <c r="D2" s="408" t="s">
+      <c r="D2" s="410" t="s">
         <v>912</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="334"/>
       <c r="B3" s="334"/>
-      <c r="C3" s="410"/>
-      <c r="D3" s="408"/>
+      <c r="C3" s="408"/>
+      <c r="D3" s="410"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="334"/>
       <c r="B4" s="334"/>
-      <c r="C4" s="410"/>
-      <c r="D4" s="408"/>
+      <c r="C4" s="408"/>
+      <c r="D4" s="410"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="334"/>
       <c r="B5" s="334"/>
-      <c r="C5" s="410"/>
-      <c r="D5" s="408"/>
+      <c r="C5" s="408"/>
+      <c r="D5" s="410"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="334"/>
       <c r="B6" s="334"/>
-      <c r="C6" s="410"/>
-      <c r="D6" s="408"/>
+      <c r="C6" s="408"/>
+      <c r="D6" s="410"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="334"/>
       <c r="B7" s="334"/>
-      <c r="C7" s="410"/>
-      <c r="D7" s="408"/>
+      <c r="C7" s="408"/>
+      <c r="D7" s="410"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="334"/>
       <c r="B8" s="334"/>
-      <c r="C8" s="410"/>
-      <c r="D8" s="408"/>
+      <c r="C8" s="408"/>
+      <c r="D8" s="410"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="334"/>
       <c r="B9" s="334"/>
-      <c r="C9" s="410"/>
-      <c r="D9" s="408"/>
+      <c r="C9" s="408"/>
+      <c r="D9" s="410"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="334"/>
       <c r="B10" s="334"/>
-      <c r="C10" s="410"/>
-      <c r="D10" s="408"/>
+      <c r="C10" s="408"/>
+      <c r="D10" s="410"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="334"/>
       <c r="B11" s="334"/>
-      <c r="C11" s="410"/>
-      <c r="D11" s="408"/>
+      <c r="C11" s="408"/>
+      <c r="D11" s="410"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="334"/>
       <c r="B12" s="334"/>
-      <c r="C12" s="410"/>
-      <c r="D12" s="408"/>
+      <c r="C12" s="408"/>
+      <c r="D12" s="410"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="334"/>
       <c r="B13" s="334"/>
-      <c r="C13" s="410"/>
-      <c r="D13" s="408"/>
+      <c r="C13" s="408"/>
+      <c r="D13" s="410"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="334"/>
       <c r="B14" s="334"/>
-      <c r="C14" s="410"/>
-      <c r="D14" s="408"/>
+      <c r="C14" s="408"/>
+      <c r="D14" s="410"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="334"/>
       <c r="B15" s="334"/>
-      <c r="C15" s="410"/>
-      <c r="D15" s="408"/>
+      <c r="C15" s="408"/>
+      <c r="D15" s="410"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="334"/>
       <c r="B16" s="334"/>
-      <c r="C16" s="410"/>
-      <c r="D16" s="408"/>
+      <c r="C16" s="408"/>
+      <c r="D16" s="410"/>
     </row>
     <row r="17" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="316"/>
       <c r="B17" s="316"/>
-      <c r="C17" s="411"/>
-      <c r="D17" s="409"/>
+      <c r="C17" s="409"/>
+      <c r="D17" s="411"/>
     </row>
     <row r="18" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="336"/>
@@ -9359,7 +9356,7 @@
       <c r="C18" s="403" t="s">
         <v>361</v>
       </c>
-      <c r="D18" s="408" t="s">
+      <c r="D18" s="410" t="s">
         <v>849</v>
       </c>
     </row>
@@ -9367,115 +9364,115 @@
       <c r="A19" s="336"/>
       <c r="B19" s="336"/>
       <c r="C19" s="403"/>
-      <c r="D19" s="408"/>
+      <c r="D19" s="410"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="336"/>
       <c r="B20" s="336"/>
       <c r="C20" s="403"/>
-      <c r="D20" s="408"/>
+      <c r="D20" s="410"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="336"/>
       <c r="B21" s="336"/>
       <c r="C21" s="403"/>
-      <c r="D21" s="408"/>
+      <c r="D21" s="410"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="336"/>
       <c r="B22" s="336"/>
       <c r="C22" s="403"/>
-      <c r="D22" s="408"/>
+      <c r="D22" s="410"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="336"/>
       <c r="B23" s="336"/>
       <c r="C23" s="403"/>
-      <c r="D23" s="408"/>
+      <c r="D23" s="410"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="336"/>
       <c r="B24" s="336"/>
       <c r="C24" s="403"/>
-      <c r="D24" s="408"/>
+      <c r="D24" s="410"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="336"/>
       <c r="B25" s="336"/>
       <c r="C25" s="403"/>
-      <c r="D25" s="408"/>
+      <c r="D25" s="410"/>
     </row>
     <row r="26" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="336"/>
       <c r="B26" s="336"/>
       <c r="C26" s="403"/>
-      <c r="D26" s="408"/>
+      <c r="D26" s="410"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="336"/>
       <c r="B27" s="336"/>
       <c r="C27" s="403"/>
-      <c r="D27" s="408"/>
+      <c r="D27" s="410"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="336"/>
       <c r="B28" s="336"/>
       <c r="C28" s="403"/>
-      <c r="D28" s="408"/>
+      <c r="D28" s="410"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="336"/>
       <c r="B29" s="336"/>
       <c r="C29" s="403"/>
-      <c r="D29" s="408"/>
+      <c r="D29" s="410"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="336"/>
       <c r="B30" s="336"/>
       <c r="C30" s="403"/>
-      <c r="D30" s="408"/>
+      <c r="D30" s="410"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="336"/>
       <c r="B31" s="336"/>
       <c r="C31" s="403"/>
-      <c r="D31" s="408"/>
+      <c r="D31" s="410"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="336"/>
       <c r="B32" s="336"/>
       <c r="C32" s="403"/>
-      <c r="D32" s="408"/>
+      <c r="D32" s="410"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="336"/>
       <c r="B33" s="336"/>
       <c r="C33" s="403"/>
-      <c r="D33" s="408"/>
+      <c r="D33" s="410"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="336"/>
       <c r="B34" s="336"/>
       <c r="C34" s="403"/>
-      <c r="D34" s="408"/>
+      <c r="D34" s="410"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="336"/>
       <c r="B35" s="336"/>
       <c r="C35" s="403"/>
-      <c r="D35" s="408"/>
+      <c r="D35" s="410"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="336"/>
       <c r="B36" s="336"/>
       <c r="C36" s="403"/>
-      <c r="D36" s="408"/>
+      <c r="D36" s="410"/>
     </row>
     <row r="37" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="317"/>
       <c r="B37" s="317"/>
       <c r="C37" s="404"/>
-      <c r="D37" s="409"/>
+      <c r="D37" s="411"/>
     </row>
     <row r="38" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="335"/>
@@ -9483,7 +9480,7 @@
       <c r="C38" s="403" t="s">
         <v>850</v>
       </c>
-      <c r="D38" s="408" t="s">
+      <c r="D38" s="410" t="s">
         <v>851</v>
       </c>
     </row>
@@ -9491,115 +9488,115 @@
       <c r="A39" s="335"/>
       <c r="B39" s="335"/>
       <c r="C39" s="403"/>
-      <c r="D39" s="408"/>
+      <c r="D39" s="410"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="335"/>
       <c r="B40" s="335"/>
       <c r="C40" s="403"/>
-      <c r="D40" s="408"/>
+      <c r="D40" s="410"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="335"/>
       <c r="B41" s="335"/>
       <c r="C41" s="403"/>
-      <c r="D41" s="408"/>
+      <c r="D41" s="410"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="335"/>
       <c r="B42" s="335"/>
       <c r="C42" s="403"/>
-      <c r="D42" s="408"/>
+      <c r="D42" s="410"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="335"/>
       <c r="B43" s="335"/>
       <c r="C43" s="403"/>
-      <c r="D43" s="408"/>
+      <c r="D43" s="410"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="335"/>
       <c r="B44" s="335"/>
       <c r="C44" s="403"/>
-      <c r="D44" s="408"/>
+      <c r="D44" s="410"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="335"/>
       <c r="B45" s="335"/>
       <c r="C45" s="403"/>
-      <c r="D45" s="408"/>
+      <c r="D45" s="410"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="335"/>
       <c r="B46" s="335"/>
       <c r="C46" s="403"/>
-      <c r="D46" s="408"/>
+      <c r="D46" s="410"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="335"/>
       <c r="B47" s="335"/>
       <c r="C47" s="403"/>
-      <c r="D47" s="408"/>
+      <c r="D47" s="410"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="335"/>
       <c r="B48" s="335"/>
       <c r="C48" s="403"/>
-      <c r="D48" s="408"/>
+      <c r="D48" s="410"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="335"/>
       <c r="B49" s="335"/>
       <c r="C49" s="403"/>
-      <c r="D49" s="408"/>
+      <c r="D49" s="410"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="335"/>
       <c r="B50" s="335"/>
       <c r="C50" s="403"/>
-      <c r="D50" s="408"/>
+      <c r="D50" s="410"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="335"/>
       <c r="B51" s="335"/>
       <c r="C51" s="403"/>
-      <c r="D51" s="408"/>
+      <c r="D51" s="410"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="335"/>
       <c r="B52" s="335"/>
       <c r="C52" s="403"/>
-      <c r="D52" s="408"/>
+      <c r="D52" s="410"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="335"/>
       <c r="B53" s="335"/>
       <c r="C53" s="403"/>
-      <c r="D53" s="408"/>
+      <c r="D53" s="410"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="335"/>
       <c r="B54" s="335"/>
       <c r="C54" s="403"/>
-      <c r="D54" s="408"/>
+      <c r="D54" s="410"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="335"/>
       <c r="B55" s="335"/>
       <c r="C55" s="403"/>
-      <c r="D55" s="408"/>
+      <c r="D55" s="410"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="335"/>
       <c r="B56" s="335"/>
       <c r="C56" s="403"/>
-      <c r="D56" s="408"/>
+      <c r="D56" s="410"/>
     </row>
     <row r="57" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="318"/>
       <c r="B57" s="318"/>
       <c r="C57" s="404"/>
-      <c r="D57" s="409"/>
+      <c r="D57" s="411"/>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="337"/>
@@ -9607,7 +9604,7 @@
       <c r="C58" s="403" t="s">
         <v>852</v>
       </c>
-      <c r="D58" s="408" t="s">
+      <c r="D58" s="410" t="s">
         <v>853</v>
       </c>
     </row>
@@ -9615,85 +9612,85 @@
       <c r="A59" s="337"/>
       <c r="B59" s="337"/>
       <c r="C59" s="403"/>
-      <c r="D59" s="408"/>
+      <c r="D59" s="410"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="337"/>
       <c r="B60" s="337"/>
       <c r="C60" s="403"/>
-      <c r="D60" s="408"/>
+      <c r="D60" s="410"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="337"/>
       <c r="B61" s="337"/>
       <c r="C61" s="403"/>
-      <c r="D61" s="408"/>
+      <c r="D61" s="410"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="337"/>
       <c r="B62" s="337"/>
       <c r="C62" s="403"/>
-      <c r="D62" s="408"/>
+      <c r="D62" s="410"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="337"/>
       <c r="B63" s="337"/>
       <c r="C63" s="403"/>
-      <c r="D63" s="408"/>
+      <c r="D63" s="410"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="337"/>
       <c r="B64" s="337"/>
       <c r="C64" s="403"/>
-      <c r="D64" s="408"/>
+      <c r="D64" s="410"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="337"/>
       <c r="B65" s="337"/>
       <c r="C65" s="403"/>
-      <c r="D65" s="408"/>
+      <c r="D65" s="410"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="337"/>
       <c r="B66" s="337"/>
       <c r="C66" s="403"/>
-      <c r="D66" s="408"/>
+      <c r="D66" s="410"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="337"/>
       <c r="B67" s="337"/>
       <c r="C67" s="403"/>
-      <c r="D67" s="408"/>
+      <c r="D67" s="410"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="337"/>
       <c r="B68" s="337"/>
       <c r="C68" s="403"/>
-      <c r="D68" s="408"/>
+      <c r="D68" s="410"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="337"/>
       <c r="B69" s="337"/>
       <c r="C69" s="403"/>
-      <c r="D69" s="408"/>
+      <c r="D69" s="410"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="337"/>
       <c r="B70" s="337"/>
       <c r="C70" s="403"/>
-      <c r="D70" s="408"/>
+      <c r="D70" s="410"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="337"/>
       <c r="B71" s="337"/>
       <c r="C71" s="403"/>
-      <c r="D71" s="408"/>
+      <c r="D71" s="410"/>
     </row>
     <row r="72" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="319"/>
       <c r="B72" s="319"/>
       <c r="C72" s="404"/>
-      <c r="D72" s="409"/>
+      <c r="D72" s="411"/>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="339"/>
@@ -9701,7 +9698,7 @@
       <c r="C73" s="403" t="s">
         <v>854</v>
       </c>
-      <c r="D73" s="408" t="s">
+      <c r="D73" s="410" t="s">
         <v>855</v>
       </c>
     </row>
@@ -9709,97 +9706,97 @@
       <c r="A74" s="339"/>
       <c r="B74" s="339"/>
       <c r="C74" s="403"/>
-      <c r="D74" s="408"/>
+      <c r="D74" s="410"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="339"/>
       <c r="B75" s="339"/>
       <c r="C75" s="403"/>
-      <c r="D75" s="408"/>
+      <c r="D75" s="410"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="339"/>
       <c r="B76" s="339"/>
       <c r="C76" s="403"/>
-      <c r="D76" s="408"/>
+      <c r="D76" s="410"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="339"/>
       <c r="B77" s="339"/>
       <c r="C77" s="403"/>
-      <c r="D77" s="408"/>
+      <c r="D77" s="410"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="339"/>
       <c r="B78" s="339"/>
       <c r="C78" s="403"/>
-      <c r="D78" s="408"/>
+      <c r="D78" s="410"/>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="339"/>
       <c r="B79" s="339"/>
       <c r="C79" s="403"/>
-      <c r="D79" s="408"/>
+      <c r="D79" s="410"/>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="339"/>
       <c r="B80" s="339"/>
       <c r="C80" s="403"/>
-      <c r="D80" s="408"/>
+      <c r="D80" s="410"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="339"/>
       <c r="B81" s="339"/>
       <c r="C81" s="403"/>
-      <c r="D81" s="408"/>
+      <c r="D81" s="410"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="339"/>
       <c r="B82" s="339"/>
       <c r="C82" s="403"/>
-      <c r="D82" s="408"/>
+      <c r="D82" s="410"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="339"/>
       <c r="B83" s="339"/>
       <c r="C83" s="403"/>
-      <c r="D83" s="408"/>
+      <c r="D83" s="410"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="339"/>
       <c r="B84" s="339"/>
       <c r="C84" s="403"/>
-      <c r="D84" s="408"/>
+      <c r="D84" s="410"/>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="339"/>
       <c r="B85" s="339"/>
       <c r="C85" s="403"/>
-      <c r="D85" s="408"/>
+      <c r="D85" s="410"/>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="339"/>
       <c r="B86" s="339"/>
       <c r="C86" s="403"/>
-      <c r="D86" s="408"/>
+      <c r="D86" s="410"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="339"/>
       <c r="B87" s="339"/>
       <c r="C87" s="403"/>
-      <c r="D87" s="408"/>
+      <c r="D87" s="410"/>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="339"/>
       <c r="B88" s="339"/>
       <c r="C88" s="403"/>
-      <c r="D88" s="408"/>
+      <c r="D88" s="410"/>
     </row>
     <row r="89" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="320"/>
       <c r="B89" s="320"/>
       <c r="C89" s="404"/>
-      <c r="D89" s="409"/>
+      <c r="D89" s="411"/>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="338"/>
@@ -9807,7 +9804,7 @@
       <c r="C90" s="403" t="s">
         <v>856</v>
       </c>
-      <c r="D90" s="408" t="s">
+      <c r="D90" s="410" t="s">
         <v>857</v>
       </c>
     </row>
@@ -9815,49 +9812,49 @@
       <c r="A91" s="338"/>
       <c r="B91" s="338"/>
       <c r="C91" s="403"/>
-      <c r="D91" s="408"/>
+      <c r="D91" s="410"/>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="338"/>
       <c r="B92" s="338"/>
       <c r="C92" s="403"/>
-      <c r="D92" s="408"/>
+      <c r="D92" s="410"/>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="338"/>
       <c r="B93" s="338"/>
       <c r="C93" s="403"/>
-      <c r="D93" s="408"/>
+      <c r="D93" s="410"/>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="338"/>
       <c r="B94" s="338"/>
       <c r="C94" s="403"/>
-      <c r="D94" s="408"/>
+      <c r="D94" s="410"/>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="338"/>
       <c r="B95" s="338"/>
       <c r="C95" s="403"/>
-      <c r="D95" s="408"/>
+      <c r="D95" s="410"/>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="338"/>
       <c r="B96" s="338"/>
       <c r="C96" s="403"/>
-      <c r="D96" s="408"/>
+      <c r="D96" s="410"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="338"/>
       <c r="B97" s="338"/>
       <c r="C97" s="403"/>
-      <c r="D97" s="408"/>
+      <c r="D97" s="410"/>
     </row>
     <row r="98" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="321"/>
       <c r="B98" s="321"/>
       <c r="C98" s="404"/>
-      <c r="D98" s="409"/>
+      <c r="D98" s="411"/>
     </row>
     <row r="99" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="340"/>
@@ -9865,7 +9862,7 @@
       <c r="C99" s="406" t="s">
         <v>858</v>
       </c>
-      <c r="D99" s="408" t="s">
+      <c r="D99" s="410" t="s">
         <v>859</v>
       </c>
     </row>
@@ -9873,73 +9870,73 @@
       <c r="A100" s="340"/>
       <c r="B100" s="340"/>
       <c r="C100" s="406"/>
-      <c r="D100" s="408"/>
+      <c r="D100" s="410"/>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="340"/>
       <c r="B101" s="340"/>
       <c r="C101" s="406"/>
-      <c r="D101" s="408"/>
+      <c r="D101" s="410"/>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="340"/>
       <c r="B102" s="340"/>
       <c r="C102" s="406"/>
-      <c r="D102" s="408"/>
+      <c r="D102" s="410"/>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="340"/>
       <c r="B103" s="340"/>
       <c r="C103" s="406"/>
-      <c r="D103" s="408"/>
+      <c r="D103" s="410"/>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="340"/>
       <c r="B104" s="340"/>
       <c r="C104" s="406"/>
-      <c r="D104" s="408"/>
+      <c r="D104" s="410"/>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="340"/>
       <c r="B105" s="340"/>
       <c r="C105" s="406"/>
-      <c r="D105" s="408"/>
+      <c r="D105" s="410"/>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="340"/>
       <c r="B106" s="340"/>
       <c r="C106" s="406"/>
-      <c r="D106" s="408"/>
+      <c r="D106" s="410"/>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="340"/>
       <c r="B107" s="340"/>
       <c r="C107" s="406"/>
-      <c r="D107" s="408"/>
+      <c r="D107" s="410"/>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="340"/>
       <c r="B108" s="340"/>
       <c r="C108" s="406"/>
-      <c r="D108" s="408"/>
+      <c r="D108" s="410"/>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="340"/>
       <c r="B109" s="340"/>
       <c r="C109" s="406"/>
-      <c r="D109" s="408"/>
+      <c r="D109" s="410"/>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="340"/>
       <c r="B110" s="340"/>
       <c r="C110" s="406"/>
-      <c r="D110" s="408"/>
+      <c r="D110" s="410"/>
     </row>
     <row r="111" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A111" s="322"/>
       <c r="B111" s="322"/>
       <c r="C111" s="407"/>
-      <c r="D111" s="409"/>
+      <c r="D111" s="411"/>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="336"/>
@@ -9947,7 +9944,7 @@
       <c r="C112" s="403" t="s">
         <v>860</v>
       </c>
-      <c r="D112" s="408" t="s">
+      <c r="D112" s="410" t="s">
         <v>861</v>
       </c>
     </row>
@@ -9955,67 +9952,67 @@
       <c r="A113" s="336"/>
       <c r="B113" s="336"/>
       <c r="C113" s="403"/>
-      <c r="D113" s="408"/>
+      <c r="D113" s="410"/>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="336"/>
       <c r="B114" s="336"/>
       <c r="C114" s="403"/>
-      <c r="D114" s="408"/>
+      <c r="D114" s="410"/>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="336"/>
       <c r="B115" s="336"/>
       <c r="C115" s="403"/>
-      <c r="D115" s="408"/>
+      <c r="D115" s="410"/>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="336"/>
       <c r="B116" s="336"/>
       <c r="C116" s="403"/>
-      <c r="D116" s="408"/>
+      <c r="D116" s="410"/>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="336"/>
       <c r="B117" s="336"/>
       <c r="C117" s="403"/>
-      <c r="D117" s="408"/>
+      <c r="D117" s="410"/>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="336"/>
       <c r="B118" s="336"/>
       <c r="C118" s="403"/>
-      <c r="D118" s="408"/>
+      <c r="D118" s="410"/>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="336"/>
       <c r="B119" s="336"/>
       <c r="C119" s="403"/>
-      <c r="D119" s="408"/>
+      <c r="D119" s="410"/>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="336"/>
       <c r="B120" s="336"/>
       <c r="C120" s="403"/>
-      <c r="D120" s="408"/>
+      <c r="D120" s="410"/>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="336"/>
       <c r="B121" s="336"/>
       <c r="C121" s="403"/>
-      <c r="D121" s="408"/>
+      <c r="D121" s="410"/>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="336"/>
       <c r="B122" s="336"/>
       <c r="C122" s="403"/>
-      <c r="D122" s="408"/>
+      <c r="D122" s="410"/>
     </row>
     <row r="123" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A123" s="317"/>
       <c r="B123" s="317"/>
       <c r="C123" s="404"/>
-      <c r="D123" s="409"/>
+      <c r="D123" s="411"/>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="335"/>
@@ -10023,7 +10020,7 @@
       <c r="C124" s="403" t="s">
         <v>862</v>
       </c>
-      <c r="D124" s="408" t="s">
+      <c r="D124" s="410" t="s">
         <v>863</v>
       </c>
     </row>
@@ -10031,31 +10028,31 @@
       <c r="A125" s="335"/>
       <c r="B125" s="335"/>
       <c r="C125" s="403"/>
-      <c r="D125" s="408"/>
+      <c r="D125" s="410"/>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="335"/>
       <c r="B126" s="335"/>
       <c r="C126" s="403"/>
-      <c r="D126" s="408"/>
+      <c r="D126" s="410"/>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="335"/>
       <c r="B127" s="335"/>
       <c r="C127" s="403"/>
-      <c r="D127" s="408"/>
+      <c r="D127" s="410"/>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="335"/>
       <c r="B128" s="335"/>
       <c r="C128" s="403"/>
-      <c r="D128" s="408"/>
+      <c r="D128" s="410"/>
     </row>
     <row r="129" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A129" s="318"/>
       <c r="B129" s="318"/>
       <c r="C129" s="404"/>
-      <c r="D129" s="409"/>
+      <c r="D129" s="411"/>
     </row>
     <row r="130" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="33"/>
@@ -10063,7 +10060,7 @@
       <c r="C130" s="403" t="s">
         <v>864</v>
       </c>
-      <c r="D130" s="408" t="s">
+      <c r="D130" s="410" t="s">
         <v>865</v>
       </c>
     </row>
@@ -10071,19 +10068,19 @@
       <c r="A131" s="33"/>
       <c r="B131" s="33"/>
       <c r="C131" s="403"/>
-      <c r="D131" s="408"/>
+      <c r="D131" s="410"/>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="33"/>
       <c r="B132" s="33"/>
       <c r="C132" s="403"/>
-      <c r="D132" s="408"/>
+      <c r="D132" s="410"/>
     </row>
     <row r="133" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A133" s="323"/>
       <c r="B133" s="323"/>
       <c r="C133" s="404"/>
-      <c r="D133" s="409"/>
+      <c r="D133" s="411"/>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="339"/>
@@ -10091,7 +10088,7 @@
       <c r="C134" s="403" t="s">
         <v>866</v>
       </c>
-      <c r="D134" s="408" t="s">
+      <c r="D134" s="410" t="s">
         <v>867</v>
       </c>
     </row>
@@ -10099,103 +10096,103 @@
       <c r="A135" s="339"/>
       <c r="B135" s="339"/>
       <c r="C135" s="403"/>
-      <c r="D135" s="408"/>
+      <c r="D135" s="410"/>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="339"/>
       <c r="B136" s="339"/>
       <c r="C136" s="403"/>
-      <c r="D136" s="408"/>
+      <c r="D136" s="410"/>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="339"/>
       <c r="B137" s="339"/>
       <c r="C137" s="403"/>
-      <c r="D137" s="408"/>
+      <c r="D137" s="410"/>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="339"/>
       <c r="B138" s="339"/>
       <c r="C138" s="403"/>
-      <c r="D138" s="408"/>
+      <c r="D138" s="410"/>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="339"/>
       <c r="B139" s="339"/>
       <c r="C139" s="403"/>
-      <c r="D139" s="408"/>
+      <c r="D139" s="410"/>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="339"/>
       <c r="B140" s="339"/>
       <c r="C140" s="403"/>
-      <c r="D140" s="408"/>
+      <c r="D140" s="410"/>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="339"/>
       <c r="B141" s="339"/>
       <c r="C141" s="403"/>
-      <c r="D141" s="408"/>
+      <c r="D141" s="410"/>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="339"/>
       <c r="B142" s="339"/>
       <c r="C142" s="403"/>
-      <c r="D142" s="408"/>
+      <c r="D142" s="410"/>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="339"/>
       <c r="B143" s="339"/>
       <c r="C143" s="403"/>
-      <c r="D143" s="408"/>
+      <c r="D143" s="410"/>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="339"/>
       <c r="B144" s="339"/>
       <c r="C144" s="403"/>
-      <c r="D144" s="408"/>
+      <c r="D144" s="410"/>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="339"/>
       <c r="B145" s="339"/>
       <c r="C145" s="403"/>
-      <c r="D145" s="408"/>
+      <c r="D145" s="410"/>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="339"/>
       <c r="B146" s="339"/>
       <c r="C146" s="403"/>
-      <c r="D146" s="408"/>
+      <c r="D146" s="410"/>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="339"/>
       <c r="B147" s="339"/>
       <c r="C147" s="403"/>
-      <c r="D147" s="408"/>
+      <c r="D147" s="410"/>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="339"/>
       <c r="B148" s="339"/>
       <c r="C148" s="403"/>
-      <c r="D148" s="408"/>
+      <c r="D148" s="410"/>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="339"/>
       <c r="B149" s="339"/>
       <c r="C149" s="403"/>
-      <c r="D149" s="408"/>
+      <c r="D149" s="410"/>
     </row>
     <row r="150" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="339"/>
       <c r="B150" s="339"/>
       <c r="C150" s="403"/>
-      <c r="D150" s="408"/>
+      <c r="D150" s="410"/>
     </row>
     <row r="151" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A151" s="320"/>
       <c r="B151" s="320"/>
       <c r="C151" s="404"/>
-      <c r="D151" s="409"/>
+      <c r="D151" s="411"/>
     </row>
     <row r="152" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="341"/>
@@ -10203,7 +10200,7 @@
       <c r="C152" s="403" t="s">
         <v>868</v>
       </c>
-      <c r="D152" s="408" t="s">
+      <c r="D152" s="410" t="s">
         <v>869</v>
       </c>
     </row>
@@ -10211,47 +10208,47 @@
       <c r="A153" s="341"/>
       <c r="B153" s="341"/>
       <c r="C153" s="403"/>
-      <c r="D153" s="408"/>
+      <c r="D153" s="410"/>
     </row>
     <row r="154" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="341"/>
       <c r="B154" s="341"/>
       <c r="C154" s="403"/>
-      <c r="D154" s="408"/>
+      <c r="D154" s="410"/>
     </row>
     <row r="155" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A155" s="324"/>
       <c r="B155" s="324"/>
       <c r="C155" s="404"/>
-      <c r="D155" s="409"/>
+      <c r="D155" s="411"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="24">
+    <mergeCell ref="C130:C133"/>
+    <mergeCell ref="D130:D133"/>
+    <mergeCell ref="C134:C151"/>
+    <mergeCell ref="D134:D151"/>
+    <mergeCell ref="C152:C155"/>
+    <mergeCell ref="D152:D155"/>
+    <mergeCell ref="C99:C111"/>
+    <mergeCell ref="D99:D111"/>
+    <mergeCell ref="C112:C123"/>
+    <mergeCell ref="D112:D123"/>
+    <mergeCell ref="C124:C129"/>
+    <mergeCell ref="D124:D129"/>
+    <mergeCell ref="C58:C72"/>
+    <mergeCell ref="D58:D72"/>
+    <mergeCell ref="C73:C89"/>
+    <mergeCell ref="D73:D89"/>
+    <mergeCell ref="C90:C98"/>
+    <mergeCell ref="D90:D98"/>
     <mergeCell ref="C2:C17"/>
     <mergeCell ref="D2:D17"/>
     <mergeCell ref="C18:C37"/>
     <mergeCell ref="D18:D37"/>
     <mergeCell ref="C38:C57"/>
     <mergeCell ref="D38:D57"/>
-    <mergeCell ref="C58:C72"/>
-    <mergeCell ref="D58:D72"/>
-    <mergeCell ref="C73:C89"/>
-    <mergeCell ref="D73:D89"/>
-    <mergeCell ref="C90:C98"/>
-    <mergeCell ref="D90:D98"/>
-    <mergeCell ref="C99:C111"/>
-    <mergeCell ref="D99:D111"/>
-    <mergeCell ref="C112:C123"/>
-    <mergeCell ref="D112:D123"/>
-    <mergeCell ref="C124:C129"/>
-    <mergeCell ref="D124:D129"/>
-    <mergeCell ref="C130:C133"/>
-    <mergeCell ref="D130:D133"/>
-    <mergeCell ref="C134:C151"/>
-    <mergeCell ref="D134:D151"/>
-    <mergeCell ref="C152:C155"/>
-    <mergeCell ref="D152:D155"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -54844,25 +54841,25 @@
     </row>
     <row r="4" spans="1:73" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="118"/>
-      <c r="B4" s="412"/>
-      <c r="C4" s="412"/>
-      <c r="D4" s="412"/>
-      <c r="E4" s="412"/>
-      <c r="F4" s="412"/>
-      <c r="G4" s="412"/>
-      <c r="H4" s="412"/>
-      <c r="I4" s="412"/>
-      <c r="J4" s="412"/>
-      <c r="K4" s="412"/>
-      <c r="L4" s="412"/>
-      <c r="M4" s="412"/>
-      <c r="N4" s="412"/>
-      <c r="O4" s="412"/>
-      <c r="P4" s="412"/>
-      <c r="Q4" s="412"/>
-      <c r="R4" s="412"/>
-      <c r="S4" s="412"/>
-      <c r="T4" s="412"/>
+      <c r="B4" s="117"/>
+      <c r="C4" s="117"/>
+      <c r="D4" s="118"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="119"/>
+      <c r="G4" s="119"/>
+      <c r="H4" s="119"/>
+      <c r="I4" s="119"/>
+      <c r="J4" s="119"/>
+      <c r="K4" s="119"/>
+      <c r="L4" s="119"/>
+      <c r="M4" s="119"/>
+      <c r="N4" s="119"/>
+      <c r="O4" s="120"/>
+      <c r="P4" s="119"/>
+      <c r="Q4" s="119"/>
+      <c r="R4" s="119"/>
+      <c r="S4" s="119"/>
+      <c r="T4" s="119"/>
       <c r="U4" s="121"/>
       <c r="V4" s="122"/>
       <c r="W4" s="122"/>
@@ -54919,25 +54916,25 @@
     </row>
     <row r="5" spans="1:73" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="118"/>
-      <c r="B5" s="412"/>
-      <c r="C5" s="412"/>
-      <c r="D5" s="412"/>
-      <c r="E5" s="412"/>
-      <c r="F5" s="412"/>
-      <c r="G5" s="412"/>
-      <c r="H5" s="412"/>
-      <c r="I5" s="412"/>
-      <c r="J5" s="412"/>
-      <c r="K5" s="412"/>
-      <c r="L5" s="412"/>
-      <c r="M5" s="412"/>
-      <c r="N5" s="412"/>
-      <c r="O5" s="412"/>
-      <c r="P5" s="412"/>
-      <c r="Q5" s="412"/>
-      <c r="R5" s="412"/>
-      <c r="S5" s="412"/>
-      <c r="T5" s="412"/>
+      <c r="B5" s="117"/>
+      <c r="C5" s="117"/>
+      <c r="D5" s="118"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="119"/>
+      <c r="G5" s="119"/>
+      <c r="H5" s="119"/>
+      <c r="I5" s="119"/>
+      <c r="J5" s="119"/>
+      <c r="K5" s="119"/>
+      <c r="L5" s="119"/>
+      <c r="M5" s="119"/>
+      <c r="N5" s="119"/>
+      <c r="O5" s="120"/>
+      <c r="P5" s="119"/>
+      <c r="Q5" s="119"/>
+      <c r="R5" s="119"/>
+      <c r="S5" s="119"/>
+      <c r="T5" s="119"/>
       <c r="U5" s="121"/>
       <c r="V5" s="122"/>
       <c r="W5" s="122"/>
@@ -54994,25 +54991,25 @@
     </row>
     <row r="6" spans="1:73" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="118"/>
-      <c r="B6" s="412"/>
-      <c r="C6" s="412"/>
-      <c r="D6" s="412"/>
-      <c r="E6" s="412"/>
-      <c r="F6" s="412"/>
-      <c r="G6" s="412"/>
-      <c r="H6" s="412"/>
-      <c r="I6" s="412"/>
-      <c r="J6" s="412"/>
-      <c r="K6" s="412"/>
-      <c r="L6" s="412"/>
-      <c r="M6" s="412"/>
-      <c r="N6" s="412"/>
-      <c r="O6" s="412"/>
-      <c r="P6" s="412"/>
-      <c r="Q6" s="412"/>
-      <c r="R6" s="412"/>
-      <c r="S6" s="412"/>
-      <c r="T6" s="412"/>
+      <c r="B6" s="117"/>
+      <c r="C6" s="117"/>
+      <c r="D6" s="118"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="119"/>
+      <c r="G6" s="119"/>
+      <c r="H6" s="119"/>
+      <c r="I6" s="119"/>
+      <c r="J6" s="119"/>
+      <c r="K6" s="119"/>
+      <c r="L6" s="119"/>
+      <c r="M6" s="119"/>
+      <c r="N6" s="119"/>
+      <c r="O6" s="120"/>
+      <c r="P6" s="119"/>
+      <c r="Q6" s="119"/>
+      <c r="R6" s="119"/>
+      <c r="S6" s="119"/>
+      <c r="T6" s="119"/>
       <c r="U6" s="121"/>
       <c r="V6" s="122"/>
       <c r="W6" s="122"/>
@@ -55069,25 +55066,25 @@
     </row>
     <row r="7" spans="1:73" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="118"/>
-      <c r="B7" s="412"/>
-      <c r="C7" s="412"/>
-      <c r="D7" s="412"/>
-      <c r="E7" s="412"/>
-      <c r="F7" s="412"/>
-      <c r="G7" s="412"/>
-      <c r="H7" s="412"/>
-      <c r="I7" s="412"/>
-      <c r="J7" s="412"/>
-      <c r="K7" s="412"/>
-      <c r="L7" s="412"/>
-      <c r="M7" s="412"/>
-      <c r="N7" s="412"/>
-      <c r="O7" s="412"/>
-      <c r="P7" s="412"/>
-      <c r="Q7" s="412"/>
-      <c r="R7" s="412"/>
-      <c r="S7" s="412"/>
-      <c r="T7" s="412"/>
+      <c r="B7" s="117"/>
+      <c r="C7" s="117"/>
+      <c r="D7" s="118"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="119"/>
+      <c r="G7" s="119"/>
+      <c r="H7" s="119"/>
+      <c r="I7" s="119"/>
+      <c r="J7" s="119"/>
+      <c r="K7" s="119"/>
+      <c r="L7" s="119"/>
+      <c r="M7" s="119"/>
+      <c r="N7" s="119"/>
+      <c r="O7" s="120"/>
+      <c r="P7" s="119"/>
+      <c r="Q7" s="119"/>
+      <c r="R7" s="119"/>
+      <c r="S7" s="119"/>
+      <c r="T7" s="119"/>
       <c r="U7" s="121"/>
       <c r="V7" s="122"/>
       <c r="W7" s="122"/>
@@ -55144,25 +55141,25 @@
     </row>
     <row r="8" spans="1:73" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="118"/>
-      <c r="B8" s="412"/>
-      <c r="C8" s="412"/>
-      <c r="D8" s="412"/>
-      <c r="E8" s="412"/>
-      <c r="F8" s="412"/>
-      <c r="G8" s="412"/>
-      <c r="H8" s="412"/>
-      <c r="I8" s="412"/>
-      <c r="J8" s="412"/>
-      <c r="K8" s="412"/>
-      <c r="L8" s="412"/>
-      <c r="M8" s="412"/>
-      <c r="N8" s="412"/>
-      <c r="O8" s="412"/>
-      <c r="P8" s="412"/>
-      <c r="Q8" s="412"/>
-      <c r="R8" s="412"/>
-      <c r="S8" s="412"/>
-      <c r="T8" s="412"/>
+      <c r="B8" s="117"/>
+      <c r="C8" s="117"/>
+      <c r="D8" s="118"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="119"/>
+      <c r="G8" s="119"/>
+      <c r="H8" s="119"/>
+      <c r="I8" s="119"/>
+      <c r="J8" s="119"/>
+      <c r="K8" s="119"/>
+      <c r="L8" s="119"/>
+      <c r="M8" s="119"/>
+      <c r="N8" s="119"/>
+      <c r="O8" s="120"/>
+      <c r="P8" s="119"/>
+      <c r="Q8" s="119"/>
+      <c r="R8" s="119"/>
+      <c r="S8" s="119"/>
+      <c r="T8" s="119"/>
       <c r="U8" s="121"/>
       <c r="V8" s="122"/>
       <c r="W8" s="122"/>
@@ -55219,25 +55216,25 @@
     </row>
     <row r="9" spans="1:73" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="118"/>
-      <c r="B9" s="412"/>
-      <c r="C9" s="412"/>
-      <c r="D9" s="412"/>
-      <c r="E9" s="412"/>
-      <c r="F9" s="412"/>
-      <c r="G9" s="412"/>
-      <c r="H9" s="412"/>
-      <c r="I9" s="412"/>
-      <c r="J9" s="412"/>
-      <c r="K9" s="412"/>
-      <c r="L9" s="412"/>
-      <c r="M9" s="412"/>
-      <c r="N9" s="412"/>
-      <c r="O9" s="412"/>
-      <c r="P9" s="412"/>
-      <c r="Q9" s="412"/>
-      <c r="R9" s="412"/>
-      <c r="S9" s="412"/>
-      <c r="T9" s="412"/>
+      <c r="B9" s="117"/>
+      <c r="C9" s="117"/>
+      <c r="D9" s="118"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="119"/>
+      <c r="G9" s="119"/>
+      <c r="H9" s="119"/>
+      <c r="I9" s="119"/>
+      <c r="J9" s="119"/>
+      <c r="K9" s="119"/>
+      <c r="L9" s="119"/>
+      <c r="M9" s="119"/>
+      <c r="N9" s="119"/>
+      <c r="O9" s="120"/>
+      <c r="P9" s="119"/>
+      <c r="Q9" s="119"/>
+      <c r="R9" s="119"/>
+      <c r="S9" s="119"/>
+      <c r="T9" s="119"/>
       <c r="U9" s="121"/>
       <c r="V9" s="122"/>
       <c r="W9" s="122"/>
@@ -55308,7 +55305,7 @@
       <c r="M10" s="119"/>
       <c r="N10" s="119"/>
       <c r="O10" s="120"/>
-      <c r="P10" s="24"/>
+      <c r="P10" s="119"/>
       <c r="Q10" s="119"/>
       <c r="R10" s="119"/>
       <c r="S10" s="119"/>
@@ -55523,18 +55520,18 @@
       <c r="C13" s="117"/>
       <c r="D13" s="118"/>
       <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="24"/>
-      <c r="I13" s="24"/>
-      <c r="J13" s="24"/>
-      <c r="K13" s="24"/>
-      <c r="L13" s="24"/>
-      <c r="M13" s="24"/>
+      <c r="F13" s="119"/>
+      <c r="G13" s="119"/>
+      <c r="H13" s="119"/>
+      <c r="I13" s="119"/>
+      <c r="J13" s="119"/>
+      <c r="K13" s="119"/>
+      <c r="L13" s="119"/>
+      <c r="M13" s="119"/>
       <c r="N13" s="119"/>
       <c r="O13" s="120"/>
-      <c r="P13" s="24"/>
-      <c r="Q13" s="24"/>
+      <c r="P13" s="119"/>
+      <c r="Q13" s="119"/>
       <c r="R13" s="119"/>
       <c r="S13" s="119"/>
       <c r="T13" s="119"/>
@@ -55598,18 +55595,18 @@
       <c r="C14" s="117"/>
       <c r="D14" s="118"/>
       <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="24"/>
-      <c r="I14" s="24"/>
-      <c r="J14" s="24"/>
-      <c r="K14" s="24"/>
-      <c r="L14" s="24"/>
-      <c r="M14" s="24"/>
+      <c r="F14" s="119"/>
+      <c r="G14" s="119"/>
+      <c r="H14" s="119"/>
+      <c r="I14" s="119"/>
+      <c r="J14" s="119"/>
+      <c r="K14" s="119"/>
+      <c r="L14" s="119"/>
+      <c r="M14" s="119"/>
       <c r="N14" s="119"/>
       <c r="O14" s="120"/>
-      <c r="P14" s="24"/>
-      <c r="Q14" s="24"/>
+      <c r="P14" s="119"/>
+      <c r="Q14" s="119"/>
       <c r="R14" s="119"/>
       <c r="S14" s="119"/>
       <c r="T14" s="119"/>
@@ -55673,18 +55670,18 @@
       <c r="C15" s="117"/>
       <c r="D15" s="118"/>
       <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="24"/>
-      <c r="J15" s="24"/>
-      <c r="K15" s="24"/>
-      <c r="L15" s="24"/>
-      <c r="M15" s="24"/>
+      <c r="F15" s="119"/>
+      <c r="G15" s="119"/>
+      <c r="H15" s="119"/>
+      <c r="I15" s="119"/>
+      <c r="J15" s="119"/>
+      <c r="K15" s="119"/>
+      <c r="L15" s="119"/>
+      <c r="M15" s="119"/>
       <c r="N15" s="119"/>
       <c r="O15" s="120"/>
-      <c r="P15" s="24"/>
-      <c r="Q15" s="24"/>
+      <c r="P15" s="119"/>
+      <c r="Q15" s="119"/>
       <c r="R15" s="119"/>
       <c r="S15" s="119"/>
       <c r="T15" s="119"/>
@@ -55748,18 +55745,18 @@
       <c r="C16" s="117"/>
       <c r="D16" s="118"/>
       <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="24"/>
-      <c r="I16" s="24"/>
-      <c r="J16" s="24"/>
-      <c r="K16" s="24"/>
-      <c r="L16" s="24"/>
-      <c r="M16" s="24"/>
+      <c r="F16" s="119"/>
+      <c r="G16" s="119"/>
+      <c r="H16" s="119"/>
+      <c r="I16" s="119"/>
+      <c r="J16" s="119"/>
+      <c r="K16" s="119"/>
+      <c r="L16" s="119"/>
+      <c r="M16" s="119"/>
       <c r="N16" s="119"/>
       <c r="O16" s="120"/>
-      <c r="P16" s="24"/>
-      <c r="Q16" s="24"/>
+      <c r="P16" s="119"/>
+      <c r="Q16" s="119"/>
       <c r="R16" s="119"/>
       <c r="S16" s="119"/>
       <c r="T16" s="119"/>
@@ -55823,18 +55820,18 @@
       <c r="C17" s="117"/>
       <c r="D17" s="118"/>
       <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="24"/>
-      <c r="I17" s="24"/>
-      <c r="J17" s="24"/>
-      <c r="K17" s="24"/>
-      <c r="L17" s="24"/>
-      <c r="M17" s="24"/>
+      <c r="F17" s="119"/>
+      <c r="G17" s="119"/>
+      <c r="H17" s="119"/>
+      <c r="I17" s="119"/>
+      <c r="J17" s="119"/>
+      <c r="K17" s="119"/>
+      <c r="L17" s="119"/>
+      <c r="M17" s="119"/>
       <c r="N17" s="119"/>
       <c r="O17" s="120"/>
-      <c r="P17" s="24"/>
-      <c r="Q17" s="24"/>
+      <c r="P17" s="119"/>
+      <c r="Q17" s="119"/>
       <c r="R17" s="119"/>
       <c r="S17" s="119"/>
       <c r="T17" s="119"/>
@@ -55895,21 +55892,21 @@
     <row r="18" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A18" s="118"/>
       <c r="B18" s="117"/>
-      <c r="C18" s="381"/>
+      <c r="C18" s="117"/>
       <c r="D18" s="118"/>
       <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="24"/>
-      <c r="J18" s="24"/>
-      <c r="K18" s="24"/>
-      <c r="L18" s="24"/>
-      <c r="M18" s="24"/>
+      <c r="F18" s="119"/>
+      <c r="G18" s="119"/>
+      <c r="H18" s="119"/>
+      <c r="I18" s="119"/>
+      <c r="J18" s="119"/>
+      <c r="K18" s="119"/>
+      <c r="L18" s="119"/>
+      <c r="M18" s="119"/>
       <c r="N18" s="119"/>
       <c r="O18" s="120"/>
-      <c r="P18" s="24"/>
-      <c r="Q18" s="24"/>
+      <c r="P18" s="119"/>
+      <c r="Q18" s="119"/>
       <c r="R18" s="119"/>
       <c r="S18" s="119"/>
       <c r="T18" s="119"/>
@@ -55973,18 +55970,18 @@
       <c r="C19" s="117"/>
       <c r="D19" s="118"/>
       <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="24"/>
-      <c r="K19" s="24"/>
-      <c r="L19" s="24"/>
-      <c r="M19" s="24"/>
-      <c r="N19" s="120"/>
+      <c r="F19" s="119"/>
+      <c r="G19" s="119"/>
+      <c r="H19" s="119"/>
+      <c r="I19" s="119"/>
+      <c r="J19" s="119"/>
+      <c r="K19" s="119"/>
+      <c r="L19" s="119"/>
+      <c r="M19" s="119"/>
+      <c r="N19" s="119"/>
       <c r="O19" s="120"/>
-      <c r="P19" s="24"/>
-      <c r="Q19" s="24"/>
+      <c r="P19" s="119"/>
+      <c r="Q19" s="119"/>
       <c r="R19" s="119"/>
       <c r="S19" s="119"/>
       <c r="T19" s="119"/>
@@ -56048,18 +56045,18 @@
       <c r="C20" s="117"/>
       <c r="D20" s="118"/>
       <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
-      <c r="I20" s="24"/>
-      <c r="J20" s="24"/>
-      <c r="K20" s="24"/>
-      <c r="L20" s="24"/>
-      <c r="M20" s="24"/>
-      <c r="N20" s="120"/>
+      <c r="F20" s="119"/>
+      <c r="G20" s="119"/>
+      <c r="H20" s="119"/>
+      <c r="I20" s="119"/>
+      <c r="J20" s="119"/>
+      <c r="K20" s="119"/>
+      <c r="L20" s="119"/>
+      <c r="M20" s="119"/>
+      <c r="N20" s="119"/>
       <c r="O20" s="120"/>
-      <c r="P20" s="24"/>
-      <c r="Q20" s="24"/>
+      <c r="P20" s="119"/>
+      <c r="Q20" s="119"/>
       <c r="R20" s="119"/>
       <c r="S20" s="119"/>
       <c r="T20" s="119"/>
@@ -56123,18 +56120,18 @@
       <c r="C21" s="117"/>
       <c r="D21" s="118"/>
       <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="24"/>
-      <c r="I21" s="24"/>
-      <c r="J21" s="24"/>
-      <c r="K21" s="24"/>
-      <c r="L21" s="24"/>
-      <c r="M21" s="24"/>
+      <c r="F21" s="119"/>
+      <c r="G21" s="119"/>
+      <c r="H21" s="119"/>
+      <c r="I21" s="119"/>
+      <c r="J21" s="119"/>
+      <c r="K21" s="119"/>
+      <c r="L21" s="119"/>
+      <c r="M21" s="119"/>
       <c r="N21" s="119"/>
       <c r="O21" s="120"/>
-      <c r="P21" s="24"/>
-      <c r="Q21" s="24"/>
+      <c r="P21" s="119"/>
+      <c r="Q21" s="119"/>
       <c r="R21" s="119"/>
       <c r="S21" s="119"/>
       <c r="T21" s="119"/>
@@ -56198,18 +56195,18 @@
       <c r="C22" s="117"/>
       <c r="D22" s="118"/>
       <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="24"/>
-      <c r="I22" s="24"/>
-      <c r="J22" s="24"/>
-      <c r="K22" s="24"/>
-      <c r="L22" s="24"/>
-      <c r="M22" s="24"/>
+      <c r="F22" s="119"/>
+      <c r="G22" s="119"/>
+      <c r="H22" s="119"/>
+      <c r="I22" s="119"/>
+      <c r="J22" s="119"/>
+      <c r="K22" s="119"/>
+      <c r="L22" s="119"/>
+      <c r="M22" s="119"/>
       <c r="N22" s="119"/>
       <c r="O22" s="120"/>
-      <c r="P22" s="24"/>
-      <c r="Q22" s="24"/>
+      <c r="P22" s="119"/>
+      <c r="Q22" s="119"/>
       <c r="R22" s="119"/>
       <c r="S22" s="119"/>
       <c r="T22" s="119"/>
@@ -56273,18 +56270,18 @@
       <c r="C23" s="117"/>
       <c r="D23" s="118"/>
       <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="24"/>
-      <c r="I23" s="24"/>
-      <c r="J23" s="24"/>
-      <c r="K23" s="24"/>
-      <c r="L23" s="24"/>
-      <c r="M23" s="24"/>
+      <c r="F23" s="119"/>
+      <c r="G23" s="119"/>
+      <c r="H23" s="119"/>
+      <c r="I23" s="119"/>
+      <c r="J23" s="119"/>
+      <c r="K23" s="119"/>
+      <c r="L23" s="119"/>
+      <c r="M23" s="119"/>
       <c r="N23" s="119"/>
       <c r="O23" s="120"/>
-      <c r="P23" s="24"/>
-      <c r="Q23" s="24"/>
+      <c r="P23" s="119"/>
+      <c r="Q23" s="119"/>
       <c r="R23" s="119"/>
       <c r="S23" s="119"/>
       <c r="T23" s="119"/>
@@ -56348,18 +56345,18 @@
       <c r="C24" s="117"/>
       <c r="D24" s="118"/>
       <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="24"/>
-      <c r="I24" s="24"/>
-      <c r="J24" s="24"/>
-      <c r="K24" s="24"/>
-      <c r="L24" s="24"/>
-      <c r="M24" s="24"/>
-      <c r="N24" s="120"/>
+      <c r="F24" s="119"/>
+      <c r="G24" s="119"/>
+      <c r="H24" s="119"/>
+      <c r="I24" s="119"/>
+      <c r="J24" s="119"/>
+      <c r="K24" s="119"/>
+      <c r="L24" s="119"/>
+      <c r="M24" s="119"/>
+      <c r="N24" s="119"/>
       <c r="O24" s="120"/>
-      <c r="P24" s="24"/>
-      <c r="Q24" s="24"/>
+      <c r="P24" s="119"/>
+      <c r="Q24" s="119"/>
       <c r="R24" s="119"/>
       <c r="S24" s="119"/>
       <c r="T24" s="119"/>
@@ -56423,18 +56420,18 @@
       <c r="C25" s="117"/>
       <c r="D25" s="118"/>
       <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
-      <c r="G25" s="24"/>
-      <c r="H25" s="24"/>
-      <c r="I25" s="24"/>
-      <c r="J25" s="24"/>
-      <c r="K25" s="24"/>
-      <c r="L25" s="24"/>
-      <c r="M25" s="24"/>
-      <c r="N25" s="120"/>
+      <c r="F25" s="119"/>
+      <c r="G25" s="119"/>
+      <c r="H25" s="119"/>
+      <c r="I25" s="119"/>
+      <c r="J25" s="119"/>
+      <c r="K25" s="119"/>
+      <c r="L25" s="119"/>
+      <c r="M25" s="119"/>
+      <c r="N25" s="119"/>
       <c r="O25" s="120"/>
-      <c r="P25" s="24"/>
-      <c r="Q25" s="24"/>
+      <c r="P25" s="119"/>
+      <c r="Q25" s="119"/>
       <c r="R25" s="119"/>
       <c r="S25" s="119"/>
       <c r="T25" s="119"/>
@@ -56498,18 +56495,18 @@
       <c r="C26" s="117"/>
       <c r="D26" s="118"/>
       <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="24"/>
-      <c r="H26" s="24"/>
-      <c r="I26" s="24"/>
-      <c r="J26" s="24"/>
-      <c r="K26" s="24"/>
-      <c r="L26" s="24"/>
-      <c r="M26" s="24"/>
-      <c r="N26" s="120"/>
+      <c r="F26" s="119"/>
+      <c r="G26" s="119"/>
+      <c r="H26" s="119"/>
+      <c r="I26" s="119"/>
+      <c r="J26" s="119"/>
+      <c r="K26" s="119"/>
+      <c r="L26" s="119"/>
+      <c r="M26" s="119"/>
+      <c r="N26" s="119"/>
       <c r="O26" s="120"/>
-      <c r="P26" s="24"/>
-      <c r="Q26" s="24"/>
+      <c r="P26" s="119"/>
+      <c r="Q26" s="119"/>
       <c r="R26" s="119"/>
       <c r="S26" s="119"/>
       <c r="T26" s="119"/>
@@ -56573,18 +56570,18 @@
       <c r="C27" s="117"/>
       <c r="D27" s="118"/>
       <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
-      <c r="G27" s="24"/>
-      <c r="H27" s="24"/>
-      <c r="I27" s="24"/>
-      <c r="J27" s="24"/>
-      <c r="K27" s="24"/>
-      <c r="L27" s="24"/>
-      <c r="M27" s="24"/>
-      <c r="N27" s="120"/>
+      <c r="F27" s="119"/>
+      <c r="G27" s="119"/>
+      <c r="H27" s="119"/>
+      <c r="I27" s="119"/>
+      <c r="J27" s="119"/>
+      <c r="K27" s="119"/>
+      <c r="L27" s="119"/>
+      <c r="M27" s="119"/>
+      <c r="N27" s="119"/>
       <c r="O27" s="120"/>
-      <c r="P27" s="24"/>
-      <c r="Q27" s="24"/>
+      <c r="P27" s="119"/>
+      <c r="Q27" s="119"/>
       <c r="R27" s="119"/>
       <c r="S27" s="119"/>
       <c r="T27" s="119"/>
@@ -56648,18 +56645,18 @@
       <c r="C28" s="117"/>
       <c r="D28" s="118"/>
       <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
-      <c r="G28" s="24"/>
-      <c r="H28" s="24"/>
-      <c r="I28" s="24"/>
-      <c r="J28" s="24"/>
-      <c r="K28" s="24"/>
-      <c r="L28" s="24"/>
-      <c r="M28" s="24"/>
+      <c r="F28" s="119"/>
+      <c r="G28" s="119"/>
+      <c r="H28" s="119"/>
+      <c r="I28" s="119"/>
+      <c r="J28" s="119"/>
+      <c r="K28" s="119"/>
+      <c r="L28" s="119"/>
+      <c r="M28" s="119"/>
       <c r="N28" s="119"/>
       <c r="O28" s="120"/>
-      <c r="P28" s="24"/>
-      <c r="Q28" s="24"/>
+      <c r="P28" s="119"/>
+      <c r="Q28" s="119"/>
       <c r="R28" s="119"/>
       <c r="S28" s="119"/>
       <c r="T28" s="119"/>
@@ -56723,18 +56720,18 @@
       <c r="C29" s="117"/>
       <c r="D29" s="118"/>
       <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="24"/>
-      <c r="H29" s="24"/>
-      <c r="I29" s="24"/>
-      <c r="J29" s="24"/>
-      <c r="K29" s="24"/>
-      <c r="L29" s="24"/>
-      <c r="M29" s="24"/>
+      <c r="F29" s="119"/>
+      <c r="G29" s="119"/>
+      <c r="H29" s="119"/>
+      <c r="I29" s="119"/>
+      <c r="J29" s="119"/>
+      <c r="K29" s="119"/>
+      <c r="L29" s="119"/>
+      <c r="M29" s="119"/>
       <c r="N29" s="119"/>
       <c r="O29" s="120"/>
-      <c r="P29" s="24"/>
-      <c r="Q29" s="24"/>
+      <c r="P29" s="119"/>
+      <c r="Q29" s="119"/>
       <c r="R29" s="119"/>
       <c r="S29" s="119"/>
       <c r="T29" s="119"/>
@@ -67586,12 +67583,6 @@
   </sheetData>
   <autoFilter ref="A2:BQ178" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <mergeCells count="15">
-    <mergeCell ref="AH1:AK1"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="E1:U1"/>
-    <mergeCell ref="V1:Y1"/>
-    <mergeCell ref="Z1:AC1"/>
-    <mergeCell ref="AD1:AG1"/>
     <mergeCell ref="BJ1:BM1"/>
     <mergeCell ref="BN1:BQ1"/>
     <mergeCell ref="BR1:BU1"/>
@@ -67601,6 +67592,12 @@
     <mergeCell ref="AX1:BA1"/>
     <mergeCell ref="BB1:BE1"/>
     <mergeCell ref="BF1:BI1"/>
+    <mergeCell ref="AH1:AK1"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="E1:U1"/>
+    <mergeCell ref="V1:Y1"/>
+    <mergeCell ref="Z1:AC1"/>
+    <mergeCell ref="AD1:AG1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -67636,19 +67633,19 @@
           <x14:formula1>
             <xm:f>datavalidation!$B$1:$B$8</xm:f>
           </x14:formula1>
-          <xm:sqref>O3 O10:O1048576</xm:sqref>
+          <xm:sqref>O3:O1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0500-000005000000}">
           <x14:formula1>
             <xm:f>datavalidation!$C$1:$C$8</xm:f>
           </x14:formula1>
-          <xm:sqref>N3 N10:N1048576</xm:sqref>
+          <xm:sqref>N3:N1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0500-000006000000}">
           <x14:formula1>
             <xm:f>datavalidation!$E$1:$E$2</xm:f>
           </x14:formula1>
-          <xm:sqref>B10:C186 B3:C3</xm:sqref>
+          <xm:sqref>B3:C186</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -77939,6 +77936,13 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C58:C60"/>
+    <mergeCell ref="C54:C57"/>
+    <mergeCell ref="C2:C11"/>
+    <mergeCell ref="C12:C17"/>
+    <mergeCell ref="C18:C28"/>
+    <mergeCell ref="C44:C53"/>
+    <mergeCell ref="C29:C43"/>
     <mergeCell ref="C163:C176"/>
     <mergeCell ref="C61:C70"/>
     <mergeCell ref="C71:C94"/>
@@ -77946,13 +77950,6 @@
     <mergeCell ref="C99:C108"/>
     <mergeCell ref="C109:C115"/>
     <mergeCell ref="C116:C162"/>
-    <mergeCell ref="C58:C60"/>
-    <mergeCell ref="C54:C57"/>
-    <mergeCell ref="C2:C11"/>
-    <mergeCell ref="C12:C17"/>
-    <mergeCell ref="C18:C28"/>
-    <mergeCell ref="C44:C53"/>
-    <mergeCell ref="C29:C43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -77960,6 +77957,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="107e75b3-53cc-4838-92d2-ebc011bd4832">
@@ -77968,15 +77974,6 @@
     <TaxCatchAll xmlns="888ccf44-0d39-41a2-ab17-f7efb2bf6977" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -78229,6 +78226,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74B21D61-7BBD-4BD3-A9A5-1E8F98F2F686}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2288FB7-E85A-4FE8-9E7A-FE572FF16064}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
@@ -78241,14 +78246,6 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="888ccf44-0d39-41a2-ab17-f7efb2bf6977"/>
     <ds:schemaRef ds:uri="107e75b3-53cc-4838-92d2-ebc011bd4832"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74B21D61-7BBD-4BD3-A9A5-1E8F98F2F686}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>